<commit_message>
Upload files via local
</commit_message>
<xml_diff>
--- a/Portfolio Analysis/Data/Trades.xlsx
+++ b/Portfolio Analysis/Data/Trades.xlsx
@@ -1,23 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kathe\Documents\PowerBI\Portfolio Performance &amp; Attribution\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kathe\Documents\PowerBI\Portfolio Analysis\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D220506-FFE2-43B4-A447-FC6B86C47F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E04C90-A53D-4352-AA6B-909A5C0C3D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{6D4F6618-3E67-4D9F-9EFF-4FAD3B04FDC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="86">
   <si>
     <t>BUY</t>
   </si>
@@ -322,6 +319,18 @@
   <si>
     <t>WCN</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GREAT WEST LIFECO INC</t>
+  </si>
+  <si>
+    <t>IGM FINANCIAL INC</t>
+  </si>
+  <si>
+    <t>GWO</t>
+  </si>
+  <si>
+    <t>IGM</t>
   </si>
 </sst>
 </file>
@@ -370,26 +379,23 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -410,40 +416,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Sheet1"/>
-      <sheetName val="SIAS Asset Detail"/>
-      <sheetName val="Sheet2"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="305">
-          <cell r="G305">
-            <v>490</v>
-          </cell>
-          <cell r="P305">
-            <v>52914</v>
-          </cell>
-        </row>
-        <row r="731">
-          <cell r="P731">
-            <v>54738</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -763,10 +735,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B15A0E-17B0-4347-BDC6-DEF3F26C7164}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.5" customWidth="1"/>
+    <col min="2" max="2" width="11.08203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.4140625" bestFit="1" customWidth="1"/>
@@ -808,7 +780,7 @@
       </c>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>35</v>
       </c>
@@ -839,41 +811,42 @@
         <v>190786.82</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="2">
+        <v>45322</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="2">
+        <v>46041</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="3">
+        <v>970</v>
+      </c>
+      <c r="I3" s="3">
+        <v>93.473699999999994</v>
+      </c>
+      <c r="J3" s="3">
+        <f>H3*I3</f>
+        <v>90669.488999999987</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>0</v>
-      </c>
-      <c r="B3" s="2">
-        <v>45382</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="3">
-        <v>490</v>
-      </c>
-      <c r="I3" s="7">
-        <f>'[1]SIAS Asset Detail'!P305/'[1]SIAS Asset Detail'!G305</f>
-        <v>107.98775510204082</v>
-      </c>
-      <c r="J3" s="3">
-        <f t="shared" ref="J3:J33" si="0">H3*I3</f>
-        <v>52914</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
       </c>
       <c r="B4" s="2">
         <v>45382</v>
@@ -882,27 +855,27 @@
         <v>20</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="H4" s="3">
-        <v>146</v>
-      </c>
-      <c r="I4" s="3">
-        <v>204.91150684931517</v>
+        <v>490</v>
+      </c>
+      <c r="I4" s="6">
+        <v>107.98775510204082</v>
       </c>
       <c r="J4" s="3">
-        <f t="shared" si="0"/>
-        <v>29917.080000000016</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <f t="shared" ref="J4:J36" si="0">H4*I4</f>
+        <v>52914</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>1</v>
       </c>
@@ -913,91 +886,91 @@
         <v>20</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H5" s="3">
-        <v>575</v>
+        <v>146</v>
       </c>
       <c r="I5" s="3">
-        <v>57.34</v>
+        <v>204.91150684931517</v>
       </c>
       <c r="J5" s="3">
         <f t="shared" si="0"/>
-        <v>32970.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>29917.080000000016</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2">
         <v>45382</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="2">
-        <v>51837</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="E6" s="3"/>
       <c r="F6" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H6" s="3">
-        <v>3760</v>
+        <v>575</v>
       </c>
       <c r="I6" s="3">
-        <v>97.6</v>
+        <v>57.34</v>
       </c>
       <c r="J6" s="3">
         <f t="shared" si="0"/>
-        <v>366976</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>32970.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="B7" s="2">
         <v>45382</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E7" s="2">
-        <v>54788</v>
-      </c>
-      <c r="F7" s="3"/>
+        <v>51837</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>2</v>
+      </c>
       <c r="G7" s="3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H7" s="3">
-        <v>198376.98997499997</v>
+        <v>3760</v>
       </c>
       <c r="I7" s="3">
-        <v>1</v>
+        <v>97.6</v>
       </c>
       <c r="J7" s="3">
         <f t="shared" si="0"/>
-        <v>198376.98997499997</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>366976</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>35</v>
       </c>
@@ -1005,34 +978,32 @@
         <v>45382</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E8" s="2">
-        <v>47959</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>49</v>
-      </c>
+        <v>54788</v>
+      </c>
+      <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="H8" s="3">
-        <v>3920</v>
+        <v>198376.98997499997</v>
       </c>
       <c r="I8" s="3">
-        <v>94.04</v>
+        <v>1</v>
       </c>
       <c r="J8" s="3">
         <f t="shared" si="0"/>
-        <v>368636.80000000005</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>198376.98997499997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2">
         <v>45382</v>
@@ -1041,29 +1012,29 @@
         <v>21</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2">
-        <v>45359</v>
+        <v>47959</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H9" s="3">
-        <v>500</v>
+        <v>3920</v>
       </c>
       <c r="I9" s="3">
-        <v>99.978999999999999</v>
+        <v>94.04</v>
       </c>
       <c r="J9" s="3">
         <f t="shared" si="0"/>
-        <v>49989.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>368636.80000000005</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
@@ -1074,29 +1045,29 @@
         <v>21</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2">
-        <v>45854</v>
+        <v>45359</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H10" s="3">
-        <v>660</v>
+        <v>500</v>
       </c>
       <c r="I10" s="3">
-        <v>100.1039</v>
+        <v>99.978999999999999</v>
       </c>
       <c r="J10" s="3">
         <f t="shared" si="0"/>
-        <v>66068.573999999993</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>49989.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>43</v>
       </c>
@@ -1106,61 +1077,61 @@
       <c r="C11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="2" t="s">
-        <v>59</v>
+      <c r="D11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2">
+        <v>45854</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H11" s="3">
-        <v>14048</v>
+        <v>660</v>
       </c>
       <c r="I11" s="3">
-        <v>28.08</v>
+        <v>100.1039</v>
       </c>
       <c r="J11" s="3">
         <f t="shared" si="0"/>
-        <v>394467.83999999997</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>66068.573999999993</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B12" s="2">
-        <v>45412</v>
+        <v>45382</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E12" s="2">
-        <v>57345</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>66</v>
+      <c r="D12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H12" s="3">
-        <v>3700</v>
+        <v>14048</v>
       </c>
       <c r="I12" s="3">
-        <v>103.8</v>
+        <v>28.08</v>
       </c>
       <c r="J12" s="3">
         <f t="shared" si="0"/>
-        <v>384060</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>394467.83999999997</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -1170,30 +1141,30 @@
       <c r="C13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>16</v>
+      <c r="D13" s="4" t="s">
+        <v>65</v>
       </c>
       <c r="E13" s="2">
-        <v>48337</v>
+        <v>57345</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H13" s="3">
-        <v>2840</v>
+        <v>3700</v>
       </c>
       <c r="I13" s="3">
-        <v>94.37</v>
+        <v>103.8</v>
       </c>
       <c r="J13" s="3">
         <f t="shared" si="0"/>
-        <v>268010.8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>384060</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -1204,29 +1175,29 @@
         <v>21</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>67</v>
+        <v>16</v>
       </c>
       <c r="E14" s="2">
         <v>48337</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H14" s="3">
-        <v>3970</v>
+        <v>2840</v>
       </c>
       <c r="I14" s="3">
-        <v>96.48</v>
+        <v>94.37</v>
       </c>
       <c r="J14" s="3">
         <f t="shared" si="0"/>
-        <v>383025.60000000003</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>268010.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>35</v>
       </c>
@@ -1237,62 +1208,64 @@
         <v>21</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E15" s="2">
-        <v>48359</v>
+        <v>48337</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H15" s="3">
+        <v>3970</v>
+      </c>
+      <c r="I15" s="3">
+        <v>96.48</v>
+      </c>
+      <c r="J15" s="3">
+        <f t="shared" si="0"/>
+        <v>383025.60000000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2">
+        <v>45412</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" s="2">
+        <v>48359</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H16" s="3">
         <v>2570</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I16" s="3">
         <v>86.92</v>
       </c>
-      <c r="J15" s="3">
+      <c r="J16" s="3">
         <f t="shared" si="0"/>
         <v>223384.4</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>1</v>
-      </c>
-      <c r="B16" s="2">
-        <v>45473</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H16" s="3">
-        <v>1000</v>
-      </c>
-      <c r="I16" s="3">
-        <v>64.7</v>
-      </c>
-      <c r="J16" s="3">
-        <f t="shared" si="0"/>
-        <v>64700</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>0</v>
       </c>
       <c r="B17" s="2">
         <v>45473</v>
@@ -1301,29 +1274,29 @@
         <v>20</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>25</v>
       </c>
       <c r="H17" s="3">
-        <v>545</v>
+        <v>1000</v>
       </c>
       <c r="I17" s="3">
-        <v>118.13</v>
+        <v>64.7</v>
       </c>
       <c r="J17" s="3">
         <f t="shared" si="0"/>
-        <v>64380.85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>64700</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="B18" s="2">
         <v>45473</v>
@@ -1332,29 +1305,29 @@
         <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>25</v>
       </c>
       <c r="H18" s="3">
-        <v>350</v>
+        <v>545</v>
       </c>
       <c r="I18" s="3">
-        <v>146.18</v>
+        <v>118.13</v>
       </c>
       <c r="J18" s="3">
         <f t="shared" si="0"/>
-        <v>51163</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>64380.85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="B19" s="2">
         <v>45473</v>
@@ -1363,60 +1336,60 @@
         <v>20</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>25</v>
       </c>
       <c r="H19" s="3">
-        <v>605</v>
+        <v>350</v>
       </c>
       <c r="I19" s="3">
-        <v>76.59</v>
+        <v>146.18</v>
       </c>
       <c r="J19" s="3">
         <f t="shared" si="0"/>
-        <v>46336.950000000004</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>51163</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" s="2">
         <v>45473</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H20" s="3">
-        <v>14053</v>
+        <v>605</v>
       </c>
       <c r="I20" s="3">
-        <v>15.09</v>
+        <v>76.59</v>
       </c>
       <c r="J20" s="3">
         <f t="shared" si="0"/>
-        <v>212059.77</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>46336.950000000004</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="B21" s="2">
         <v>45473</v>
@@ -1425,31 +1398,27 @@
         <v>21</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="2">
-        <v>45811</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E21" s="3"/>
       <c r="F21" s="3" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="H21" s="3">
-        <f>(29808.88-20130.88)/100</f>
-        <v>96.78</v>
+        <v>14053</v>
       </c>
       <c r="I21" s="3">
-        <f>AVERAGE(99.98,100.137)</f>
-        <v>100.05850000000001</v>
+        <v>15.09</v>
       </c>
       <c r="J21" s="3">
         <f t="shared" si="0"/>
-        <v>9683.6616300000005</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>212059.77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>43</v>
       </c>
@@ -1460,29 +1429,29 @@
         <v>21</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E22" s="2">
-        <v>45446</v>
+        <v>45811</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="H22" s="3">
-        <v>2000</v>
+        <v>96.78</v>
       </c>
       <c r="I22" s="3">
-        <v>99.983199999999997</v>
+        <v>100.05850000000001</v>
       </c>
       <c r="J22" s="3">
         <f t="shared" si="0"/>
-        <v>199966.4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>9683.6616300000005</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>43</v>
       </c>
@@ -1490,32 +1459,34 @@
         <v>45473</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="E23" s="2">
+        <v>45446</v>
+      </c>
       <c r="F23" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="H23" s="3">
-        <v>3134</v>
+        <v>2000</v>
       </c>
       <c r="I23" s="3">
-        <v>46.04</v>
+        <v>99.983199999999997</v>
       </c>
       <c r="J23" s="3">
         <f t="shared" si="0"/>
-        <v>144289.35999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>199966.4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B24" s="2">
         <v>45473</v>
@@ -1524,60 +1495,58 @@
         <v>20</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>77</v>
       </c>
       <c r="H24" s="3">
+        <v>3134</v>
+      </c>
+      <c r="I24" s="3">
+        <v>46.04</v>
+      </c>
+      <c r="J24" s="3">
+        <f t="shared" si="0"/>
+        <v>144289.35999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="2">
+        <v>45473</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H25" s="3">
         <v>1567</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I25" s="3">
         <v>50.6</v>
       </c>
-      <c r="J24" s="3">
+      <c r="J25" s="3">
         <f t="shared" si="0"/>
         <v>79290.2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" s="2">
-        <v>45504</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="2">
-        <v>47324</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H25" s="3">
-        <v>1000</v>
-      </c>
-      <c r="I25" s="3">
-        <v>99.851100000000002</v>
-      </c>
-      <c r="J25" s="3">
-        <f t="shared" si="0"/>
-        <v>99851.1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>43</v>
       </c>
@@ -1587,63 +1556,63 @@
       <c r="C26" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>63</v>
+      <c r="D26" t="s">
+        <v>16</v>
       </c>
       <c r="E26" s="2">
-        <v>45502</v>
+        <v>47324</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>25</v>
       </c>
       <c r="H26" s="3">
-        <v>730</v>
+        <v>1000</v>
       </c>
       <c r="I26" s="3">
-        <v>99.8035</v>
+        <v>99.851100000000002</v>
       </c>
       <c r="J26" s="3">
         <f t="shared" si="0"/>
-        <v>72856.554999999993</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>99851.1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B27" s="2">
-        <v>45535</v>
+        <v>45504</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E27" s="2">
-        <v>50685</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>61</v>
+        <v>45502</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="H27" s="3">
-        <v>4310</v>
+        <v>730</v>
       </c>
       <c r="I27" s="3">
-        <v>88.305999999999997</v>
+        <v>99.8035</v>
       </c>
       <c r="J27" s="3">
         <f t="shared" si="0"/>
-        <v>380598.86</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>72856.554999999993</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>35</v>
       </c>
@@ -1651,32 +1620,34 @@
         <v>45535</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3" t="s">
-        <v>3</v>
+        <v>60</v>
+      </c>
+      <c r="E28" s="2">
+        <v>50685</v>
+      </c>
+      <c r="F28" t="s">
+        <v>61</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="H28" s="3">
-        <v>666</v>
+        <v>4310</v>
       </c>
       <c r="I28" s="3">
-        <v>82.275285285285278</v>
+        <v>88.305999999999997</v>
       </c>
       <c r="J28" s="3">
         <f t="shared" si="0"/>
-        <v>54795.34</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>380598.86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B29" s="2">
         <v>45535</v>
@@ -1685,29 +1656,29 @@
         <v>20</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="E29" s="3"/>
       <c r="F29" s="3" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="H29" s="3">
-        <v>2525</v>
+        <v>666</v>
       </c>
       <c r="I29" s="3">
-        <v>43.2</v>
+        <v>99.81</v>
       </c>
       <c r="J29" s="3">
         <f t="shared" si="0"/>
-        <v>109080</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>66473.460000000006</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B30" s="2">
         <v>45535</v>
@@ -1716,61 +1687,60 @@
         <v>20</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>44</v>
       </c>
       <c r="H30" s="3">
-        <v>13</v>
-      </c>
-      <c r="I30" s="7">
-        <f>'[1]SIAS Asset Detail'!P731/13</f>
-        <v>4210.6153846153848</v>
+        <v>2525</v>
+      </c>
+      <c r="I30" s="3">
+        <v>43.2</v>
       </c>
       <c r="J30" s="3">
         <f t="shared" si="0"/>
-        <v>54738</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>109080</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B31" s="2">
-        <v>45565</v>
+        <v>45535</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H31" s="3">
-        <v>867</v>
-      </c>
-      <c r="I31" s="3">
-        <v>113.33</v>
+        <v>13</v>
+      </c>
+      <c r="I31" s="6">
+        <v>4210.6153846153848</v>
       </c>
       <c r="J31" s="3">
         <f t="shared" si="0"/>
-        <v>98257.11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>54738</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B32" s="2">
         <v>45565</v>
@@ -1779,29 +1749,29 @@
         <v>20</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>42</v>
       </c>
       <c r="H32" s="3">
-        <v>985</v>
+        <v>867</v>
       </c>
       <c r="I32" s="3">
-        <v>157.435</v>
+        <v>113.33</v>
       </c>
       <c r="J32" s="3">
         <f t="shared" si="0"/>
-        <v>155073.47500000001</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>98257.11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B33" s="2">
         <v>45565</v>
@@ -1809,24 +1779,115 @@
       <c r="C33" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>80</v>
-      </c>
+      <c r="D33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="3"/>
       <c r="F33" s="3" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>42</v>
       </c>
       <c r="H33" s="3">
+        <v>985</v>
+      </c>
+      <c r="I33" s="3">
+        <v>157.435</v>
+      </c>
+      <c r="J33" s="3">
+        <f t="shared" si="0"/>
+        <v>155073.47500000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="2">
+        <v>45565</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" t="s">
+        <v>80</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H34" s="3">
         <v>443</v>
       </c>
-      <c r="I33" s="4">
+      <c r="I34">
         <v>251.95756207674944</v>
       </c>
-      <c r="J33" s="3">
+      <c r="J34" s="3">
         <f t="shared" si="0"/>
         <v>111617.2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="2">
+        <v>45565</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" t="s">
+        <v>82</v>
+      </c>
+      <c r="F35" t="s">
+        <v>84</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H35" s="3">
+        <v>1735</v>
+      </c>
+      <c r="I35" s="3">
+        <v>44.3</v>
+      </c>
+      <c r="J35" s="3">
+        <f t="shared" si="0"/>
+        <v>76860.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="2">
+        <v>45565</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" t="s">
+        <v>83</v>
+      </c>
+      <c r="F36" t="s">
+        <v>85</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H36" s="3">
+        <v>690</v>
+      </c>
+      <c r="I36" s="3">
+        <v>39.68</v>
+      </c>
+      <c r="J36" s="3">
+        <f t="shared" si="0"/>
+        <v>27379.200000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>